<commit_message>
Update to the Excel options sheet for heat pump targeting.
</commit_message>
<xml_diff>
--- a/Excel_Version/Data_input_template.xlsx
+++ b/Excel_Version/Data_input_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timothyw/Github Local/OpenPinch/Excel_Version/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{306F13BF-845E-024A-B736-201033D91622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7797D68A-CD01-D64B-851C-A42661309E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" activeTab="2" xr2:uid="{BB0ED48D-3077-FB46-BBC1-F820D8E91AAE}"/>
   </bookViews>
@@ -20,13 +20,12 @@
   <externalReferences>
     <externalReference r:id="rId4"/>
     <externalReference r:id="rId5"/>
-    <externalReference r:id="rId6"/>
   </externalReferences>
   <definedNames>
     <definedName name="a">#REF!</definedName>
     <definedName name="b">#REF!</definedName>
     <definedName name="c_0">#REF!</definedName>
-    <definedName name="configuration" localSheetId="2">Options!$A$1:$B$44</definedName>
+    <definedName name="configuration" localSheetId="2">Options!$A$1:$B$46</definedName>
     <definedName name="Dev_01">#REF!</definedName>
     <definedName name="Dev_02">#REF!</definedName>
     <definedName name="Dev_03">#REF!</definedName>
@@ -43,7 +42,7 @@
     <definedName name="h_per_year">#REF!</definedName>
     <definedName name="i">#REF!</definedName>
     <definedName name="n">#REF!</definedName>
-    <definedName name="ProductionRate">[3]Summary!$C$8</definedName>
+    <definedName name="ProductionRate">[2]Summary!$C$8</definedName>
   </definedNames>
   <calcPr calcId="181029" iterate="1" iterateCount="5000" calcOnSave="0"/>
   <extLst>
@@ -68,7 +67,7 @@
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
   <connection id="1" xr16:uid="{4A486B45-271F-D245-BBE4-08B881A71805}" name="configuration" type="6" refreshedVersion="8" background="1" saveData="1">
-    <textPr codePage="10000" sourceFile="/Users/timothyw/Github Local/OpenPinch/OpenPinch/lib/configuration.txt" delimiter=":">
+    <textPr sourceFile="/Users/timothyw/Github Local/OpenPinch/OpenPinch/lib/configuration.txt" delimiter=":">
       <textFields count="2">
         <textField/>
         <textField/>
@@ -79,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="145">
   <si>
     <t>Process Zone</t>
   </si>
@@ -594,6 +593,12 @@
   </si>
   <si>
     <t>SERV_LIFE</t>
+  </si>
+  <si>
+    <t>DO_REFRIGERANT_SORT</t>
+  </si>
+  <si>
+    <t>DT_CASCADE_HX</t>
   </si>
 </sst>
 </file>
@@ -699,13 +704,13 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -779,72 +784,6 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Test Data"/>
-      <sheetName val="Summary"/>
-      <sheetName val="Stream Data"/>
-      <sheetName val="Record"/>
-      <sheetName val="Utility Data"/>
-      <sheetName val="PT"/>
-      <sheetName val="CC"/>
-      <sheetName val="SCC"/>
-      <sheetName val="GCC"/>
-      <sheetName val="BCC"/>
-      <sheetName val="GCC (NP)"/>
-      <sheetName val="GCC (Ext)"/>
-      <sheetName val="GCC (Act)"/>
-      <sheetName val="ETD"/>
-      <sheetName val="HSDT"/>
-      <sheetName val="TSP"/>
-      <sheetName val="NLC"/>
-      <sheetName val="xBCC"/>
-      <sheetName val="xGCC"/>
-      <sheetName val="xNLC"/>
-      <sheetName val="Multi-output"/>
-      <sheetName val="Options"/>
-      <sheetName val="License"/>
-      <sheetName val="Input HEN"/>
-      <sheetName val="Grid"/>
-      <sheetName val="Example_ART_Input"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -1231,10 +1170,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1254,8 +1193,8 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
       <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
@@ -2768,10 +2707,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="12" t="s">
         <v>11</v>
       </c>
       <c r="C1" s="5" t="s">
@@ -2791,8 +2730,8 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
       <c r="C2" s="6" t="s">
         <v>7</v>
       </c>
@@ -2923,234 +2862,244 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F7EE7E0-8CC0-0B49-AC08-EF1AF9C010A9}">
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="33.83203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="12"/>
+    <col min="1" max="1" width="33.83203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="10" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="10" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="10" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="10" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="10" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="10" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="10" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="10" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="10" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="10" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="10" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="10" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="10" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="10" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="10" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="10" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="10" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="10" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="10" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="10" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="10" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="10" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="10" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="10" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A29" s="10" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A29" s="12" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A30" s="10" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A30" s="12" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A31" s="10" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A31" s="12" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A32" s="10" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A32" s="12" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A33" s="10" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A33" s="12" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A34" s="10" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A34" s="12" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A35" s="10" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A35" s="12" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A36" s="10" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A36" s="12" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A37" s="10" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A37" s="12" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A38" s="10" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A39" s="10" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A38" s="12" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A40" s="10" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A39" s="12" t="s">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A41" s="10" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A40" s="12" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A42" s="10" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A41" s="12" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A43" s="10" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A42" s="12" t="s">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A44" s="10" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A43" s="12" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A45" s="10" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A44" s="12" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A46" s="10" t="s">
         <v>142</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Minor fix to the keywords in Excel.
</commit_message>
<xml_diff>
--- a/Excel_Version/Data_input_template.xlsx
+++ b/Excel_Version/Data_input_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timothyw/Github Local/OpenPinch/Excel_Version/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7797D68A-CD01-D64B-851C-A42661309E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D94879D0-1386-AF42-AE09-52E81789603F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" activeTab="2" xr2:uid="{BB0ED48D-3077-FB46-BBC1-F820D8E91AAE}"/>
+    <workbookView xWindow="-38400" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="2" xr2:uid="{BB0ED48D-3077-FB46-BBC1-F820D8E91AAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Stream Data" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <definedName name="a">#REF!</definedName>
     <definedName name="b">#REF!</definedName>
     <definedName name="c_0">#REF!</definedName>
-    <definedName name="configuration" localSheetId="2">Options!$A$1:$B$46</definedName>
+    <definedName name="configuration" localSheetId="2">Options!$A$1:$B$47</definedName>
     <definedName name="Dev_01">#REF!</definedName>
     <definedName name="Dev_02">#REF!</definedName>
     <definedName name="Dev_03">#REF!</definedName>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="146">
   <si>
     <t>Process Zone</t>
   </si>
@@ -599,6 +599,9 @@
   </si>
   <si>
     <t>DT_CASCADE_HX</t>
+  </si>
+  <si>
+    <t>DT_HP_IHX</t>
   </si>
 </sst>
 </file>
@@ -2862,7 +2865,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F7EE7E0-8CC0-0B49-AC08-EF1AF9C010A9}">
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="33.83203125" style="10" bestFit="1" customWidth="1"/>
@@ -3060,46 +3063,51 @@
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A38" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A39" s="10" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A40" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A41" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A42" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A43" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A44" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A45" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A46" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.15">
+      <c r="A47" s="10" t="s">
         <v>142</v>
       </c>
     </row>

</xml_diff>